<commit_message>
Add Nov (25) prior-year November column support
Template (financial_template_v2_2026.xlsx):
  - BM16: 'Forecast Nov'          → 'Forecast Nov (25)'
  - BN16: 'Accrual Nov'           → 'Accrual Nov (25)'
  - BO16: 'Actual Nov'            → 'Actual Nov (25)'
  - BQ16: already 'Accrual Reversal Nov (25)' (set in previous commit)
  All four November metric columns now share the key 'Nov (25)'.

transactional_detail_reader.get_transactional_data:
  - AP12 Actuals/Reversals now emit 'Nov (25)' (shifted_num==11 gets the
    same prior-year suffix as shifted_num==0 does for Dec (25)).
  - Month-sort collector extended to also gather 'Nov (' prefixed keys,
    ordering them Nov (25) → Dec (25) → Jan → … → Dec.

template_writer:
  - month_sort_key: 'Nov (YY)' returns -1 (before Dec (25) at 0).
  - write_hierarchy Pass 1: cross-fallback added for 'Nov (25)' ↔ 'Nov'
    mismatch, mirroring the existing Dec (25) ↔ Dec fallback.
</commit_message>
<xml_diff>
--- a/data/templates/financial_template_v2_2026.xlsx
+++ b/data/templates/financial_template_v2_2026.xlsx
@@ -2939,20 +2939,20 @@
       <x:c r="BL16" s="63" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="BM16" s="52" t="s">
-        <x:v>85</x:v>
-      </x:c>
-      <x:c r="BN16" s="52" t="s">
-        <x:v>86</x:v>
-      </x:c>
-      <x:c r="BO16" s="64" t="s">
-        <x:v>87</x:v>
+      <x:c r="BM16" s="52" t="str">
+        <x:v>Forecast Nov (25)</x:v>
+      </x:c>
+      <x:c r="BN16" s="52" t="str">
+        <x:v>Accrual Nov (25)</x:v>
+      </x:c>
+      <x:c r="BO16" s="64" t="str">
+        <x:v>Actual Nov (25)</x:v>
       </x:c>
       <x:c r="BP16" s="65" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="BQ16" s="63" t="s">
-        <x:v>88</x:v>
+      <x:c r="BQ16" s="63" t="str">
+        <x:v>Accrual Reversal Nov (25)</x:v>
       </x:c>
       <x:c r="BR16" s="52" t="s">
         <x:v>89</x:v>

</xml_diff>